<commit_message>
Updated the unit of electricity price data
Updated the unit of electricity price data.
</commit_message>
<xml_diff>
--- a/data/2024_ElectricityPrice.xlsx
+++ b/data/2024_ElectricityPrice.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HuZheng\Desktop\FPV2.0\经济效益\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\FPV2.0\GlobalFPV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DFE6ECA-3CE0-4B37-B276-E4920CC287F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D7198E6-E6F9-4968-97C1-65143AD0D419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{D96AAF56-E782-46FB-B221-C838ACE2FBC1}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{D96AAF56-E782-46FB-B221-C838ACE2FBC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -467,14 +470,6 @@
     <t>Iran</t>
   </si>
   <si>
-    <t>Rprice</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Bprice</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>BMU</t>
   </si>
   <si>
@@ -915,6 +910,64 @@
   </si>
   <si>
     <t>DZA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Residential price (USD kWh</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>⁻</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>¹)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Business price (USD kWh</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>⁻</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>¹)</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -922,7 +975,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -946,6 +999,14 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="3"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1312,33 +1373,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23DE797E-4961-45EF-B0DD-2229A24F250F}">
   <dimension ref="A1:D145"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="31.6640625" customWidth="1"/>
-    <col min="2" max="2" width="20.25" customWidth="1"/>
+    <col min="2" max="2" width="20.265625" customWidth="1"/>
     <col min="4" max="4" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>143</v>
+        <v>289</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C2">
         <v>0.46200000000000002</v>
@@ -1347,23 +1408,23 @@
         <v>0.26900000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C3">
         <v>0.443</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C4">
         <v>0.42199999999999999</v>
@@ -1372,12 +1433,12 @@
         <v>0.442</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C5">
         <v>0.41299999999999998</v>
@@ -1386,12 +1447,12 @@
         <v>0.36899999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C6">
         <v>0.41</v>
@@ -1400,12 +1461,12 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C7">
         <v>0.40200000000000002</v>
@@ -1414,12 +1475,12 @@
         <v>0.28599999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C8">
         <v>0.4</v>
@@ -1428,12 +1489,12 @@
         <v>0.26200000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C9">
         <v>0.39700000000000002</v>
@@ -1442,12 +1503,12 @@
         <v>0.44500000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C10">
         <v>0.36099999999999999</v>
@@ -1456,12 +1517,12 @@
         <v>0.28399999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C11">
         <v>0.35699999999999998</v>
@@ -1470,12 +1531,12 @@
         <v>0.377</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C12">
         <v>0.35499999999999998</v>
@@ -1484,12 +1545,12 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C13">
         <v>0.35199999999999998</v>
@@ -1498,12 +1559,12 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C14">
         <v>0.33600000000000002</v>
@@ -1512,12 +1573,12 @@
         <v>0.29199999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C15">
         <v>0.33400000000000002</v>
@@ -1526,12 +1587,12 @@
         <v>0.30399999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C16">
         <v>0.32700000000000001</v>
@@ -1540,12 +1601,12 @@
         <v>0.19900000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C17">
         <v>0.314</v>
@@ -1554,12 +1615,12 @@
         <v>0.33200000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C18">
         <v>0.29499999999999998</v>
@@ -1568,12 +1629,12 @@
         <v>0.186</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C19">
         <v>0.28799999999999998</v>
@@ -1582,12 +1643,12 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C20">
         <v>0.28599999999999998</v>
@@ -1596,12 +1657,12 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C21">
         <v>0.28499999999999998</v>
@@ -1610,12 +1671,12 @@
         <v>0.24199999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C22">
         <v>0.28299999999999997</v>
@@ -1624,12 +1685,12 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C23">
         <v>0.27800000000000002</v>
@@ -1638,12 +1699,12 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C24">
         <v>0.27</v>
@@ -1652,12 +1713,12 @@
         <v>0.18099999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C25">
         <v>0.254</v>
@@ -1666,12 +1727,12 @@
         <v>0.23699999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C26">
         <v>0.25</v>
@@ -1680,12 +1741,12 @@
         <v>0.123</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C27">
         <v>0.247</v>
@@ -1694,12 +1755,12 @@
         <v>0.218</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C28">
         <v>0.246</v>
@@ -1708,12 +1769,12 @@
         <v>0.23899999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C29">
         <v>0.246</v>
@@ -1722,12 +1783,12 @@
         <v>0.20799999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C30">
         <v>0.24399999999999999</v>
@@ -1736,12 +1797,12 @@
         <v>0.24199999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C31">
         <v>0.24299999999999999</v>
@@ -1750,12 +1811,12 @@
         <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C32">
         <v>0.23400000000000001</v>
@@ -1764,12 +1825,12 @@
         <v>0.28100000000000003</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C33">
         <v>0.23100000000000001</v>
@@ -1778,23 +1839,23 @@
         <v>0.152</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C34">
         <v>0.23</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C35">
         <v>0.22900000000000001</v>
@@ -1803,12 +1864,12 @@
         <v>0.20699999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C36">
         <v>0.22900000000000001</v>
@@ -1817,12 +1878,12 @@
         <v>0.39400000000000002</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C37">
         <v>0.224</v>
@@ -1831,12 +1892,12 @@
         <v>0.29099999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C38">
         <v>0.223</v>
@@ -1845,12 +1906,12 @@
         <v>0.189</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C39">
         <v>0.22</v>
@@ -1859,12 +1920,12 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C40">
         <v>0.217</v>
@@ -1873,12 +1934,12 @@
         <v>0.157</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C41">
         <v>0.217</v>
@@ -1887,12 +1948,12 @@
         <v>0.17299999999999999</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C42">
         <v>0.21299999999999999</v>
@@ -1901,12 +1962,12 @@
         <v>0.318</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C43">
         <v>0.20899999999999999</v>
@@ -1915,12 +1976,12 @@
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C44">
         <v>0.20599999999999999</v>
@@ -1929,12 +1990,12 @@
         <v>0.153</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C45">
         <v>0.20399999999999999</v>
@@ -1943,23 +2004,23 @@
         <v>0.21099999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C46">
         <v>0.20399999999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C47">
         <v>0.20300000000000001</v>
@@ -1968,12 +2029,12 @@
         <v>0.16800000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C48">
         <v>0.20300000000000001</v>
@@ -1982,12 +2043,12 @@
         <v>0.151</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C49">
         <v>0.20300000000000001</v>
@@ -1996,12 +2057,12 @@
         <v>7.5999999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C50">
         <v>0.20100000000000001</v>
@@ -2010,12 +2071,12 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C51">
         <v>0.192</v>
@@ -2024,12 +2085,12 @@
         <v>0.17699999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C52">
         <v>0.187</v>
@@ -2038,12 +2099,12 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C53">
         <v>0.187</v>
@@ -2052,12 +2113,12 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C54">
         <v>0.186</v>
@@ -2066,12 +2127,12 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C55">
         <v>0.186</v>
@@ -2080,7 +2141,7 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -2094,23 +2155,23 @@
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C57">
         <v>0.18099999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C58">
         <v>0.17599999999999999</v>
@@ -2119,12 +2180,12 @@
         <v>0.218</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C59">
         <v>0.17499999999999999</v>
@@ -2133,12 +2194,12 @@
         <v>0.22800000000000001</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C60">
         <v>0.17399999999999999</v>
@@ -2147,12 +2208,12 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C61">
         <v>0.17199999999999999</v>
@@ -2161,12 +2222,12 @@
         <v>0.193</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C62">
         <v>0.17100000000000001</v>
@@ -2175,12 +2236,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C63">
         <v>0.16900000000000001</v>
@@ -2189,12 +2250,12 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C64">
         <v>0.16800000000000001</v>
@@ -2203,12 +2264,12 @@
         <v>8.1000000000000003E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C65">
         <v>0.16800000000000001</v>
@@ -2217,12 +2278,12 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C66">
         <v>0.16300000000000001</v>
@@ -2231,12 +2292,12 @@
         <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C67">
         <v>0.159</v>
@@ -2245,12 +2306,12 @@
         <v>0.128</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C68">
         <v>0.152</v>
@@ -2259,23 +2320,23 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C69">
         <v>0.15</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C70">
         <v>0.14599999999999999</v>
@@ -2284,12 +2345,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C71">
         <v>0.14499999999999999</v>
@@ -2298,23 +2359,23 @@
         <v>0.16200000000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C72">
         <v>0.13600000000000001</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C73">
         <v>0.13400000000000001</v>
@@ -2323,12 +2384,12 @@
         <v>0.13400000000000001</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C74">
         <v>0.129</v>
@@ -2337,12 +2398,12 @@
         <v>0.16800000000000001</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C75">
         <v>0.127</v>
@@ -2351,12 +2412,12 @@
         <v>0.22800000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C76">
         <v>0.127</v>
@@ -2365,12 +2426,12 @@
         <v>0.129</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C77">
         <v>0.127</v>
@@ -2379,12 +2440,12 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C78">
         <v>0.127</v>
@@ -2393,12 +2454,12 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C79">
         <v>0.126</v>
@@ -2407,12 +2468,12 @@
         <v>0.11600000000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C80">
         <v>0.125</v>
@@ -2421,12 +2482,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C81">
         <v>0.125</v>
@@ -2435,12 +2496,12 @@
         <v>0.23599999999999999</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C82">
         <v>0.125</v>
@@ -2449,12 +2510,12 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C83">
         <v>0.123</v>
@@ -2463,12 +2524,12 @@
         <v>0.106</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C84">
         <v>0.121</v>
@@ -2477,12 +2538,12 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C85">
         <v>0.11799999999999999</v>
@@ -2491,12 +2552,12 @@
         <v>0.108</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C86">
         <v>0.11700000000000001</v>
@@ -2505,12 +2566,12 @@
         <v>0.17399999999999999</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C87">
         <v>0.11700000000000001</v>
@@ -2519,12 +2580,12 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C88">
         <v>0.111</v>
@@ -2533,12 +2594,12 @@
         <v>0.109</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C89">
         <v>0.108</v>
@@ -2547,12 +2608,12 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C90">
         <v>0.106</v>
@@ -2561,23 +2622,23 @@
         <v>0.21099999999999999</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C91">
         <v>0.105</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C92">
         <v>0.10199999999999999</v>
@@ -2586,12 +2647,12 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C93">
         <v>9.9000000000000005E-2</v>
@@ -2600,12 +2661,12 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C94">
         <v>9.7000000000000003E-2</v>
@@ -2614,12 +2675,12 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C95">
         <v>9.6000000000000002E-2</v>
@@ -2628,12 +2689,12 @@
         <v>0.17499999999999999</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C96">
         <v>9.4E-2</v>
@@ -2642,12 +2703,12 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C97">
         <v>9.1999999999999998E-2</v>
@@ -2656,12 +2717,12 @@
         <v>7.0999999999999994E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C98">
         <v>9.0999999999999998E-2</v>
@@ -2670,12 +2731,12 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C99">
         <v>0.09</v>
@@ -2684,12 +2745,12 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C100">
         <v>8.6999999999999994E-2</v>
@@ -2698,12 +2759,12 @@
         <v>0.14599999999999999</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C101">
         <v>8.3000000000000004E-2</v>
@@ -2712,12 +2773,12 @@
         <v>0.109</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C102">
         <v>8.3000000000000004E-2</v>
@@ -2726,12 +2787,12 @@
         <v>0.17499999999999999</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C103">
         <v>0.08</v>
@@ -2740,12 +2801,12 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C104">
         <v>7.8E-2</v>
@@ -2754,12 +2815,12 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C105">
         <v>7.6999999999999999E-2</v>
@@ -2768,12 +2829,12 @@
         <v>0.126</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C106">
         <v>7.6999999999999999E-2</v>
@@ -2782,12 +2843,12 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C107">
         <v>7.5999999999999998E-2</v>
@@ -2796,12 +2857,12 @@
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C108">
         <v>7.3999999999999996E-2</v>
@@ -2810,12 +2871,12 @@
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C109">
         <v>6.9000000000000006E-2</v>
@@ -2824,12 +2885,12 @@
         <v>8.1000000000000003E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C110">
         <v>6.7000000000000004E-2</v>
@@ -2838,12 +2899,12 @@
         <v>0.114</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C111">
         <v>6.7000000000000004E-2</v>
@@ -2852,12 +2913,12 @@
         <v>0.14699999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C112">
         <v>6.7000000000000004E-2</v>
@@ -2866,12 +2927,12 @@
         <v>0.106</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C113">
         <v>6.5000000000000002E-2</v>
@@ -2880,12 +2941,12 @@
         <v>0.157</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C114">
         <v>6.4000000000000001E-2</v>
@@ -2894,12 +2955,12 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C115">
         <v>6.3E-2</v>
@@ -2908,12 +2969,12 @@
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C116">
         <v>6.2E-2</v>
@@ -2922,12 +2983,12 @@
         <v>9.9000000000000005E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C117">
         <v>5.5E-2</v>
@@ -2936,12 +2997,12 @@
         <v>7.3999999999999996E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C118">
         <v>5.5E-2</v>
@@ -2950,12 +3011,12 @@
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C119">
         <v>5.2999999999999999E-2</v>
@@ -2964,12 +3025,12 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C120">
         <v>5.0999999999999997E-2</v>
@@ -2978,12 +3039,12 @@
         <v>6.8000000000000005E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C121">
         <v>0.05</v>
@@ -2992,12 +3053,12 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" t="s">
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C122">
         <v>4.9000000000000002E-2</v>
@@ -3006,12 +3067,12 @@
         <v>0.128</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A123" t="s">
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C123">
         <v>4.8000000000000001E-2</v>
@@ -3020,12 +3081,12 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C124">
         <v>4.7E-2</v>
@@ -3034,23 +3095,23 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C125">
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B126" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C126">
         <v>4.2999999999999997E-2</v>
@@ -3059,12 +3120,12 @@
         <v>6.9000000000000006E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B127" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C127">
         <v>0.04</v>
@@ -3073,12 +3134,12 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" t="s">
         <v>125</v>
       </c>
       <c r="B128" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C128">
         <v>3.6999999999999998E-2</v>
@@ -3087,12 +3148,12 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
         <v>126</v>
       </c>
       <c r="B129" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C129">
         <v>3.5999999999999997E-2</v>
@@ -3101,12 +3162,12 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A130" t="s">
         <v>127</v>
       </c>
       <c r="B130" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C130">
         <v>3.4000000000000002E-2</v>
@@ -3115,12 +3176,12 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A131" t="s">
         <v>128</v>
       </c>
       <c r="B131" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C131">
         <v>3.2000000000000001E-2</v>
@@ -3129,23 +3190,23 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
         <v>129</v>
       </c>
       <c r="B132" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C132">
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
         <v>130</v>
       </c>
       <c r="B133" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C133">
         <v>2.8000000000000001E-2</v>
@@ -3154,12 +3215,12 @@
         <v>0.19800000000000001</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
         <v>131</v>
       </c>
       <c r="B134" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C134">
         <v>2.5999999999999999E-2</v>
@@ -3168,12 +3229,12 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A135" t="s">
         <v>132</v>
       </c>
       <c r="B135" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C135">
         <v>2.4E-2</v>
@@ -3182,12 +3243,12 @@
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" t="s">
         <v>133</v>
       </c>
       <c r="B136" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C136">
         <v>2.3E-2</v>
@@ -3196,23 +3257,23 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" t="s">
         <v>134</v>
       </c>
       <c r="B137" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C137">
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" t="s">
         <v>135</v>
       </c>
       <c r="B138" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C138">
         <v>1.4999999999999999E-2</v>
@@ -3221,12 +3282,12 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" t="s">
         <v>136</v>
       </c>
       <c r="B139" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C139">
         <v>1.4999999999999999E-2</v>
@@ -3235,12 +3296,12 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" t="s">
         <v>137</v>
       </c>
       <c r="B140" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C140">
         <v>1.4999999999999999E-2</v>
@@ -3249,12 +3310,12 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" t="s">
         <v>138</v>
       </c>
       <c r="B141" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C141">
         <v>1.4E-2</v>
@@ -3263,12 +3324,12 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" t="s">
         <v>139</v>
       </c>
       <c r="B142" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C142">
         <v>1.4E-2</v>
@@ -3277,12 +3338,12 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" t="s">
         <v>140</v>
       </c>
       <c r="B143" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C143">
         <v>7.0000000000000001E-3</v>
@@ -3291,12 +3352,12 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" t="s">
         <v>141</v>
       </c>
       <c r="B144" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C144">
         <v>6.0000000000000001E-3</v>
@@ -3305,12 +3366,12 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A145" t="s">
         <v>142</v>
       </c>
       <c r="B145" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C145">
         <v>3.0000000000000001E-3</v>

</xml_diff>